<commit_message>
stage before training 08062026
Reorganize calibration IO pipeline files and remove legacy reporting scripts.
</commit_message>
<xml_diff>
--- a/Training/Day3_Calibration/ModelBaseline5Sectorsand1Regions.xlsx
+++ b/Training/Day3_Calibration/ModelBaseline5Sectorsand1Regions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schul\Documents\GitHub\DGE-METRIC\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D5B9E7-518A-4378-AC8D-188D8EC54061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2068DCEC-E562-4B4A-8139-3ACE91F1852B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>Sheets</t>
   </si>
@@ -156,10 +156,10 @@
     <t>exo_targetIY_3_1</t>
   </si>
   <si>
-    <t>exo_lTargetInv_2_1</t>
-  </si>
-  <si>
-    <t>exo_lTargetInv_3_1</t>
+    <t>exo_ltargetIY_2_1</t>
+  </si>
+  <si>
+    <t>exo_ltargetIY_3_1</t>
   </si>
   <si>
     <t>exo_P_K_1_1</t>
@@ -213,6 +213,12 @@
     <t>exo_AI_5_1_2</t>
   </si>
   <si>
+    <t>exo_PV_1_2</t>
+  </si>
+  <si>
+    <t>exo_PVEff_1_2</t>
+  </si>
+  <si>
     <t>exo_lFDIShare_3_1</t>
   </si>
   <si>
@@ -222,40 +228,34 @@
     <t>exo_r_FDI_3_1</t>
   </si>
   <si>
+    <t>idx_PV_Res_1</t>
+  </si>
+  <si>
+    <t>exo_PV_1</t>
+  </si>
+  <si>
     <t>exo_GA_4_1</t>
   </si>
   <si>
     <t>exo_GA_5_1</t>
   </si>
   <si>
+    <t>idx_GA_4_1_plan</t>
+  </si>
+  <si>
+    <t>idx_GA_5_1_plan</t>
+  </si>
+  <si>
+    <t>idx_PV_1_plan</t>
+  </si>
+  <si>
+    <t>idx_PV_1_plan_inv</t>
+  </si>
+  <si>
     <t>exo_lAddEE_4_1</t>
   </si>
   <si>
     <t>exo_lAddEE_5_1</t>
-  </si>
-  <si>
-    <t>exo_PVEff_1_2</t>
-  </si>
-  <si>
-    <t>idx_PV_Res_1</t>
-  </si>
-  <si>
-    <t>exo_PV_1</t>
-  </si>
-  <si>
-    <t>idx_GA_4_1_plan</t>
-  </si>
-  <si>
-    <t>idx_GA_5_1_plan</t>
-  </si>
-  <si>
-    <t>idx_PV_1_plan</t>
-  </si>
-  <si>
-    <t>idx_PV_1_plan_inv</t>
-  </si>
-  <si>
-    <t>exo_PV_1_2</t>
   </si>
 </sst>
 </file>
@@ -735,42 +735,42 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM26"/>
+  <dimension ref="A1:BL26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="2.109375" customWidth="1"/>
-    <col min="18" max="18" width="14.6640625" customWidth="1"/>
-    <col min="19" max="21" width="2.109375" customWidth="1"/>
-    <col min="22" max="22" width="14.33203125" customWidth="1"/>
-    <col min="23" max="23" width="12.33203125" customWidth="1"/>
-    <col min="24" max="24" width="2.109375" customWidth="1"/>
-    <col min="25" max="26" width="12.6640625" customWidth="1"/>
-    <col min="27" max="28" width="2.109375" customWidth="1"/>
-    <col min="29" max="30" width="13.6640625" customWidth="1"/>
+    <col min="15" max="15" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="21" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="30" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="31" max="38" width="2.109375" customWidth="1"/>
     <col min="39" max="39" width="7.33203125" customWidth="1"/>
     <col min="40" max="47" width="2.109375" customWidth="1"/>
     <col min="48" max="49" width="13.6640625" customWidth="1"/>
-    <col min="50" max="50" width="2.109375" customWidth="1"/>
-    <col min="51" max="51" width="4.6640625" customWidth="1"/>
-    <col min="52" max="52" width="14.33203125" customWidth="1"/>
-    <col min="53" max="54" width="13.6640625" customWidth="1"/>
-    <col min="55" max="56" width="2.109375" customWidth="1"/>
-    <col min="58" max="58" width="13.6640625" customWidth="1"/>
-    <col min="59" max="59" width="11.6640625" customWidth="1"/>
-    <col min="60" max="60" width="14.6640625" customWidth="1"/>
-    <col min="61" max="64" width="11.6640625" customWidth="1"/>
-    <col min="65" max="65" width="8.6640625" customWidth="1"/>
+    <col min="50" max="50" width="8.6640625" customWidth="1"/>
+    <col min="51" max="51" width="13.6640625" customWidth="1"/>
+    <col min="52" max="52" width="2.109375" customWidth="1"/>
+    <col min="53" max="53" width="4.6640625" customWidth="1"/>
+    <col min="54" max="54" width="14.33203125" customWidth="1"/>
+    <col min="55" max="55" width="11.6640625" customWidth="1"/>
+    <col min="56" max="56" width="14.6640625" customWidth="1"/>
+    <col min="57" max="58" width="13.6640625" customWidth="1"/>
+    <col min="59" max="62" width="11.6640625" customWidth="1"/>
+    <col min="63" max="64" width="2.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -816,158 +816,155 @@
       <c r="O1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="BE1" t="s">
-        <v>53</v>
-      </c>
-      <c r="BF1" t="s">
+      <c r="BE1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BF1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BG1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BH1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BI1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BJ1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BK1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BL1" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
@@ -975,10 +972,10 @@
         <v>2026</v>
       </c>
       <c r="C2">
-        <v>1.3047225968583029E-2</v>
+        <v>7.2516633953202065E-3</v>
       </c>
       <c r="D2">
-        <v>2.2335684435685569E-3</v>
+        <v>1.822047269944792E-3</v>
       </c>
       <c r="E2">
         <v>1.0518321404802085</v>
@@ -1116,38 +1113,37 @@
         <v>0.02</v>
       </c>
       <c r="AX2">
-        <v>1</v>
+        <v>1.067571</v>
       </c>
       <c r="AY2">
+        <v>6.7665190508490347E-2</v>
+      </c>
+      <c r="AZ2">
+        <v>1</v>
+      </c>
+      <c r="BA2">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ2">
+      <c r="BB2">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA2">
-        <v>4.2000000000000003E-2</v>
-      </c>
-      <c r="BB2">
-        <v>2.8000000000000011E-2</v>
-      </c>
       <c r="BC2">
         <v>1</v>
       </c>
       <c r="BD2">
-        <v>1</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="BE2">
-        <f>0.01*A2</f>
-        <v>0.02</v>
+        <v>1.9E-2</v>
       </c>
       <c r="BF2">
-        <v>6.7665190508490347E-2</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="BG2">
         <v>1</v>
       </c>
       <c r="BH2">
-        <v>1.2999999999999999E-3</v>
+        <v>1</v>
       </c>
       <c r="BI2">
         <v>1</v>
@@ -1161,11 +1157,8 @@
       <c r="BL2">
         <v>1</v>
       </c>
-      <c r="BM2">
-        <v>1.067571</v>
-      </c>
     </row>
-    <row r="3" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
@@ -1173,10 +1166,10 @@
         <v>2027</v>
       </c>
       <c r="C3">
-        <v>2.5749945750924989E-2</v>
+        <v>1.4451118538174506E-2</v>
       </c>
       <c r="D3">
-        <v>4.3649794513741071E-3</v>
+        <v>3.6407807206558424E-3</v>
       </c>
       <c r="E3">
         <v>1.0496263296845247</v>
@@ -1314,56 +1307,52 @@
         <v>4.2907013246408846E-2</v>
       </c>
       <c r="AX3">
-        <v>1</v>
+        <v>1.1397600000000001</v>
       </c>
       <c r="AY3">
+        <v>0.13539852345039727</v>
+      </c>
+      <c r="AZ3">
+        <v>1</v>
+      </c>
+      <c r="BA3">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ3">
+      <c r="BB3">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA3">
-        <v>5.0599116510215397E-2</v>
-      </c>
-      <c r="BB3">
-        <v>3.3732744340143547E-2</v>
-      </c>
       <c r="BC3">
-        <v>1</v>
+        <v>2.4356709000552055</v>
       </c>
       <c r="BD3">
-        <v>1</v>
+        <v>3.1663721700717672E-3</v>
       </c>
       <c r="BE3">
-        <f t="shared" ref="BE3:BE26" si="0">0.01*A3</f>
-        <v>0.03</v>
+        <v>2.4297073440088371E-2</v>
       </c>
       <c r="BF3">
-        <v>0.13539852345039727</v>
+        <v>2.1153506350082809E-2</v>
       </c>
       <c r="BG3">
-        <v>2.4356709000552055</v>
+        <v>1.143567090005523</v>
       </c>
       <c r="BH3">
-        <v>3.1663721700717672E-3</v>
+        <v>1.1435670900055206</v>
       </c>
       <c r="BI3">
-        <v>1.143567090005523</v>
+        <v>1.1435670900055217</v>
       </c>
       <c r="BJ3">
-        <v>1.1435670900055206</v>
+        <v>2.4356709000552166</v>
       </c>
       <c r="BK3">
-        <v>1.1435670900055217</v>
+        <v>1</v>
       </c>
       <c r="BL3">
-        <v>2.4356709000552166</v>
-      </c>
-      <c r="BM3">
-        <v>1.1397600000000001</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
@@ -1371,10 +1360,10 @@
         <v>2028</v>
       </c>
       <c r="C4">
-        <v>3.797558985305842E-2</v>
+        <v>2.1599111803461721E-2</v>
       </c>
       <c r="D4">
-        <v>6.2338654224300839E-3</v>
+        <v>5.4562123841645068E-3</v>
       </c>
       <c r="E4">
         <v>1.0472087963307122</v>
@@ -1512,56 +1501,52 @@
         <v>6.9407794021680402E-2</v>
       </c>
       <c r="AX4">
-        <v>1</v>
+        <v>1.216888</v>
       </c>
       <c r="AY4">
+        <v>0.2031995860302872</v>
+      </c>
+      <c r="AZ4">
+        <v>1</v>
+      </c>
+      <c r="BA4">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ4">
+      <c r="BB4">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA4">
-        <v>6.4732744340143561E-2</v>
-      </c>
-      <c r="BB4">
-        <v>4.315516289342905E-2</v>
-      </c>
       <c r="BC4">
-        <v>1</v>
+        <v>3.9983434566537923</v>
       </c>
       <c r="BD4">
-        <v>1</v>
+        <v>5.1978464936499299E-3</v>
       </c>
       <c r="BE4">
-        <f t="shared" si="0"/>
-        <v>0.04</v>
+        <v>3.1864715626725569E-2</v>
       </c>
       <c r="BF4">
-        <v>0.2031995860302872</v>
+        <v>2.7435670900055213E-2</v>
       </c>
       <c r="BG4">
-        <v>3.9983434566537923</v>
+        <v>1.4290447266703479</v>
       </c>
       <c r="BH4">
-        <v>5.1978464936499299E-3</v>
+        <v>1.4290447266703477</v>
       </c>
       <c r="BI4">
         <v>1.4290447266703479</v>
       </c>
       <c r="BJ4">
-        <v>1.4290447266703477</v>
+        <v>3.9983434566537834</v>
       </c>
       <c r="BK4">
-        <v>1.4290447266703479</v>
+        <v>1</v>
       </c>
       <c r="BL4">
-        <v>3.9983434566537834</v>
-      </c>
-      <c r="BM4">
-        <v>1.216888</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
@@ -1569,10 +1554,10 @@
         <v>2029</v>
       </c>
       <c r="C5">
-        <v>4.9635383152666621E-2</v>
+        <v>2.8696373674223338E-2</v>
       </c>
       <c r="D5">
-        <v>7.7227935961330461E-3</v>
+        <v>7.2683542270908447E-3</v>
       </c>
       <c r="E5">
         <v>1.044547520762156</v>
@@ -1710,56 +1695,52 @@
         <v>0.11115701287280108</v>
       </c>
       <c r="AX5">
-        <v>1</v>
+        <v>1.299296</v>
       </c>
       <c r="AY5">
+        <v>0.27106781689211473</v>
+      </c>
+      <c r="AZ5">
+        <v>1</v>
+      </c>
+      <c r="BA5">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ5">
+      <c r="BB5">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA5">
-        <v>0.10203810049696271</v>
-      </c>
-      <c r="BB5">
-        <v>6.8025400331308883E-2</v>
-      </c>
       <c r="BC5">
-        <v>1</v>
+        <v>10.225289895085661</v>
       </c>
       <c r="BD5">
-        <v>1</v>
+        <v>1.3292876863611358E-2</v>
       </c>
       <c r="BE5">
-        <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>4.8938707896189829E-2</v>
       </c>
       <c r="BF5">
-        <v>0.27106781689211473</v>
+        <v>4.2630038652678184E-2</v>
       </c>
       <c r="BG5">
-        <v>10.225289895085661</v>
+        <v>2.3086692435118645</v>
       </c>
       <c r="BH5">
-        <v>1.3292876863611358E-2</v>
+        <v>2.3086692435118792</v>
       </c>
       <c r="BI5">
-        <v>2.3086692435118645</v>
+        <v>2.3086692435118721</v>
       </c>
       <c r="BJ5">
-        <v>2.3086692435118792</v>
+        <v>10.22528989508559</v>
       </c>
       <c r="BK5">
-        <v>2.3086692435118721</v>
+        <v>1</v>
       </c>
       <c r="BL5">
-        <v>10.22528989508559</v>
-      </c>
-      <c r="BM5">
-        <v>1.299296</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
@@ -1767,10 +1748,10 @@
         <v>2030</v>
       </c>
       <c r="C6">
-        <v>6.0676180938982943E-2</v>
+        <v>3.5743619189626333E-2</v>
       </c>
       <c r="D6">
-        <v>8.7792173570151281E-3</v>
+        <v>9.0772181511169E-3</v>
       </c>
       <c r="E6">
         <v>1.0416036839404668</v>
@@ -1908,56 +1889,52 @@
         <v>0.17465109009273258</v>
       </c>
       <c r="AX6">
-        <v>1</v>
+        <v>1.387348</v>
       </c>
       <c r="AY6">
+        <v>0.33900402892856984</v>
+      </c>
+      <c r="AZ6">
+        <v>1</v>
+      </c>
+      <c r="BA6">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ6">
+      <c r="BB6">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA6">
-        <v>0.17321380452788521</v>
-      </c>
-      <c r="BB6">
-        <v>0.11547586968525676</v>
-      </c>
       <c r="BC6">
-        <v>1</v>
+        <v>19.789618995030288</v>
       </c>
       <c r="BD6">
-        <v>1</v>
+        <v>2.5726504693539376E-2</v>
       </c>
       <c r="BE6">
-        <f t="shared" si="0"/>
-        <v>0.06</v>
+        <v>7.9908227498619588E-2</v>
       </c>
       <c r="BF6">
-        <v>0.33900402892856984</v>
+        <v>7.0851463279955798E-2</v>
       </c>
       <c r="BG6">
-        <v>19.789618995030288</v>
+        <v>4.0567642186637238</v>
       </c>
       <c r="BH6">
-        <v>2.5726504693539376E-2</v>
+        <v>4.0567642186637203</v>
       </c>
       <c r="BI6">
-        <v>4.0567642186637238</v>
+        <v>4.0567642186637221</v>
       </c>
       <c r="BJ6">
-        <v>4.0567642186637203</v>
+        <v>19.789618995030366</v>
       </c>
       <c r="BK6">
-        <v>4.0567642186637221</v>
+        <v>1</v>
       </c>
       <c r="BL6">
-        <v>19.789618995030366</v>
-      </c>
-      <c r="BM6">
-        <v>1.387348</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
@@ -1965,10 +1942,10 @@
         <v>2031</v>
       </c>
       <c r="C7">
-        <v>6.9155401833132513E-2</v>
+        <v>3.6024478621328009E-2</v>
       </c>
       <c r="D7">
-        <v>7.5813110606110937E-3</v>
+        <v>2.1053409197832915E-2</v>
       </c>
       <c r="E7">
         <v>1.0512000000000001</v>
@@ -2106,56 +2083,52 @@
         <v>0.15804108352638394</v>
       </c>
       <c r="AX7">
-        <v>1</v>
+        <v>1.4814369999999999</v>
       </c>
       <c r="AY7">
+        <v>0.40700858300437631</v>
+      </c>
+      <c r="AZ7">
+        <v>1</v>
+      </c>
+      <c r="BA7">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ7">
+      <c r="BB7">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA7">
-        <v>0.13891204856946143</v>
-      </c>
-      <c r="BB7">
-        <v>9.3383602555144357E-2</v>
-      </c>
       <c r="BC7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BE7">
-        <f t="shared" si="0"/>
-        <v>7.0000000000000007E-2</v>
+        <v>6.7015199413112375E-2</v>
       </c>
       <c r="BF7">
-        <v>0.40700858300437631</v>
+        <v>5.8529001474121725E-2</v>
       </c>
       <c r="BG7">
-        <v>0</v>
+        <v>3.1259499633195236</v>
       </c>
       <c r="BH7">
-        <v>0</v>
+        <v>3.1686000982747822</v>
       </c>
       <c r="BI7">
-        <v>3.1259499633195236</v>
+        <v>3.1474323578133627</v>
       </c>
       <c r="BJ7">
-        <v>3.1686000982747822</v>
+        <v>0</v>
       </c>
       <c r="BK7">
-        <v>3.1474323578133627</v>
+        <v>1</v>
       </c>
       <c r="BL7">
-        <v>0</v>
-      </c>
-      <c r="BM7">
-        <v>1.4814369999999999</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
@@ -2163,10 +2136,10 @@
         <v>2032</v>
       </c>
       <c r="C8">
-        <v>7.7465830972737945E-2</v>
+        <v>3.6305259193157122E-2</v>
       </c>
       <c r="D8">
-        <v>6.6735318838913723E-3</v>
+        <v>3.2887866844835856E-2</v>
       </c>
       <c r="E8">
         <v>1.0448229166666669</v>
@@ -2304,56 +2277,52 @@
         <v>0.1751524767154912</v>
       </c>
       <c r="AX8">
-        <v>1</v>
+        <v>1.5819810000000001</v>
       </c>
       <c r="AY8">
+        <v>0.47508009715096439</v>
+      </c>
+      <c r="AZ8">
+        <v>1</v>
+      </c>
+      <c r="BA8">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ8">
+      <c r="BB8">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA8">
-        <v>0.15494300090857754</v>
-      </c>
-      <c r="BB8">
-        <v>0.10511883655538655</v>
-      </c>
       <c r="BC8">
-        <v>1</v>
+        <v>7.2975362522140808</v>
       </c>
       <c r="BD8">
-        <v>1</v>
+        <v>9.4867971278783051E-3</v>
       </c>
       <c r="BE8">
-        <f t="shared" si="0"/>
-        <v>0.08</v>
+        <v>7.4771487552236948E-2</v>
       </c>
       <c r="BF8">
-        <v>0.47508009715096439</v>
+        <v>6.5722405705030684E-2</v>
       </c>
       <c r="BG8">
-        <v>7.2975362522140808</v>
+        <v>3.4857179720148088</v>
       </c>
       <c r="BH8">
-        <v>9.4867971278783051E-3</v>
+        <v>3.5814937136687122</v>
       </c>
       <c r="BI8">
-        <v>3.4857179720148088</v>
+        <v>3.53395913859746</v>
       </c>
       <c r="BJ8">
-        <v>3.5814937136687122</v>
+        <v>7.0127001656543353</v>
       </c>
       <c r="BK8">
-        <v>3.53395913859746</v>
+        <v>1</v>
       </c>
       <c r="BL8">
-        <v>7.0127001656543353</v>
-      </c>
-      <c r="BM8">
-        <v>1.5819810000000001</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
@@ -2361,10 +2330,10 @@
         <v>2033</v>
       </c>
       <c r="C9">
-        <v>8.5572265411138465E-2</v>
+        <v>3.6585960949386306E-2</v>
       </c>
       <c r="D9">
-        <v>6.1736674036573921E-3</v>
+        <v>4.4583906608026386E-2</v>
       </c>
       <c r="E9">
         <v>1.0385315217391304</v>
@@ -2502,56 +2471,52 @@
         <v>0.1917985604514553</v>
       </c>
       <c r="AX9">
-        <v>1</v>
+        <v>1.689427</v>
       </c>
       <c r="AY9">
+        <v>0.54322040082674306</v>
+      </c>
+      <c r="AZ9">
+        <v>1</v>
+      </c>
+      <c r="BA9">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ9">
+      <c r="BB9">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA9">
-        <v>0.17076817452148954</v>
-      </c>
-      <c r="BB9">
-        <v>0.11698924700348762</v>
-      </c>
       <c r="BC9">
-        <v>1</v>
+        <v>7.7624208090921964</v>
       </c>
       <c r="BD9">
-        <v>1</v>
+        <v>1.0091147051819856E-2</v>
       </c>
       <c r="BE9">
-        <f t="shared" si="0"/>
-        <v>0.09</v>
+        <v>8.2443353649841872E-2</v>
       </c>
       <c r="BF9">
-        <v>0.54322040082674306</v>
+        <v>7.2993796348165912E-2</v>
       </c>
       <c r="BG9">
-        <v>7.7624208090921964</v>
+        <v>3.8402096031151167</v>
       </c>
       <c r="BH9">
-        <v>1.0091147051819856E-2</v>
+        <v>3.9995864232110607</v>
       </c>
       <c r="BI9">
-        <v>3.8402096031151167</v>
+        <v>3.9204859193815573</v>
       </c>
       <c r="BJ9">
-        <v>3.9995864232110607</v>
+        <v>7.399226946438433</v>
       </c>
       <c r="BK9">
-        <v>3.9204859193815573</v>
+        <v>1</v>
       </c>
       <c r="BL9">
-        <v>7.399226946438433</v>
-      </c>
-      <c r="BM9">
-        <v>1.689427</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
@@ -2559,10 +2524,10 @@
         <v>2034</v>
       </c>
       <c r="C10">
-        <v>9.3439886466750055E-2</v>
+        <v>3.6866583934250276E-2</v>
       </c>
       <c r="D10">
-        <v>6.2014667482928418E-3</v>
+        <v>5.6144729009102688E-2</v>
       </c>
       <c r="E10">
         <v>1.0322937784090913</v>
@@ -2700,56 +2665,52 @@
         <v>0.20799287814770356</v>
       </c>
       <c r="AX10">
-        <v>1</v>
+        <v>1.8042549999999999</v>
       </c>
       <c r="AY10">
+        <v>0.61142831892488558</v>
+      </c>
+      <c r="AZ10">
+        <v>1</v>
+      </c>
+      <c r="BA10">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ10">
+      <c r="BB10">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA10">
-        <v>0.18638756940819748</v>
-      </c>
-      <c r="BB10">
-        <v>0.12899483389944752</v>
-      </c>
       <c r="BC10">
-        <v>1</v>
+        <v>8.2325044601187081</v>
       </c>
       <c r="BD10">
-        <v>1</v>
+        <v>1.0702255798154319E-2</v>
       </c>
       <c r="BE10">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
+        <v>9.0030797705927174E-2</v>
       </c>
       <c r="BF10">
-        <v>0.61142831892488558</v>
+        <v>8.0343173403527382E-2</v>
       </c>
       <c r="BG10">
-        <v>8.2325044601187081</v>
+        <v>4.1894248566204482</v>
       </c>
       <c r="BH10">
-        <v>1.0702255798154319E-2</v>
+        <v>4.4228782269018261</v>
       </c>
       <c r="BI10">
-        <v>4.1894248566204482</v>
+        <v>4.3070127001656546</v>
       </c>
       <c r="BJ10">
-        <v>4.4228782269018261</v>
+        <v>7.7857537272225308</v>
       </c>
       <c r="BK10">
-        <v>4.3070127001656546</v>
+        <v>1</v>
       </c>
       <c r="BL10">
-        <v>7.7857537272225308</v>
-      </c>
-      <c r="BM10">
-        <v>1.8042549999999999</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
@@ -2757,10 +2718,10 @@
         <v>2035</v>
       </c>
       <c r="C11">
-        <v>9.8843813186937843E-2</v>
+        <v>3.7147128191946537E-2</v>
       </c>
       <c r="D11">
-        <v>4.7120380594618747E-3</v>
+        <v>6.7573424832725548E-2</v>
       </c>
       <c r="E11">
         <v>1.0260743750000001</v>
@@ -2898,56 +2859,52 @@
         <v>0.2513941006551057</v>
       </c>
       <c r="AX11">
-        <v>1</v>
+        <v>1.9269769999999999</v>
       </c>
       <c r="AY11">
+        <v>0.67970422759671867</v>
+      </c>
+      <c r="AZ11">
+        <v>1</v>
+      </c>
+      <c r="BA11">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ11">
+      <c r="BB11">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA11">
-        <v>0.24647156511309373</v>
-      </c>
-      <c r="BB11">
-        <v>0.1730048688479302</v>
-      </c>
       <c r="BC11">
-        <v>1</v>
+        <v>20.965199360933621</v>
       </c>
       <c r="BD11">
-        <v>1</v>
+        <v>2.7254759169213705E-2</v>
       </c>
       <c r="BE11">
-        <f t="shared" si="0"/>
-        <v>0.11</v>
+        <v>0.11586012927716666</v>
       </c>
       <c r="BF11">
-        <v>0.67970422759671867</v>
+        <v>0.10615665510457509</v>
       </c>
       <c r="BG11">
-        <v>20.965199360933621</v>
+        <v>5.6787580798229165</v>
       </c>
       <c r="BH11">
-        <v>2.7254759169213705E-2</v>
+        <v>6.0771103403050057</v>
       </c>
       <c r="BI11">
-        <v>5.6787580798229165</v>
+        <v>5.8794036443953619</v>
       </c>
       <c r="BJ11">
-        <v>6.0771103403050057</v>
+        <v>20.030922142462728</v>
       </c>
       <c r="BK11">
-        <v>5.8794036443953619</v>
+        <v>1</v>
       </c>
       <c r="BL11">
-        <v>20.030922142462728</v>
-      </c>
-      <c r="BM11">
-        <v>1.9269769999999999</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
@@ -2955,10 +2912,10 @@
         <v>2036</v>
       </c>
       <c r="C12">
-        <v>0.10392542912170701</v>
+        <v>3.6585960949386091E-2</v>
       </c>
       <c r="D12">
-        <v>4.1235579114977331E-3</v>
+        <v>7.9434620090189853E-2</v>
       </c>
       <c r="E12">
         <v>1.02125</v>
@@ -3096,56 +3053,52 @@
         <v>0.23908181895024369</v>
       </c>
       <c r="AX12">
-        <v>1</v>
+        <v>2.0581420000000001</v>
       </c>
       <c r="AY12">
+        <v>0.74804815942090075</v>
+      </c>
+      <c r="AZ12">
+        <v>1</v>
+      </c>
+      <c r="BA12">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ12">
+      <c r="BB12">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA12">
-        <v>0.2170090230030001</v>
-      </c>
-      <c r="BB12">
-        <v>0.15341153703494453</v>
-      </c>
       <c r="BC12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BE12">
-        <f t="shared" si="0"/>
-        <v>0.12</v>
+        <v>0.1049524196935385</v>
       </c>
       <c r="BF12">
-        <v>0.74804815942090075</v>
+        <v>9.5275886750929503E-2</v>
       </c>
       <c r="BG12">
-        <v>0</v>
+        <v>4.8720262308461564</v>
       </c>
       <c r="BH12">
-        <v>0</v>
+        <v>5.2850591167286334</v>
       </c>
       <c r="BI12">
-        <v>4.8720262308461564</v>
+        <v>5.0800662617338483</v>
       </c>
       <c r="BJ12">
-        <v>5.2850591167286334</v>
+        <v>0</v>
       </c>
       <c r="BK12">
-        <v>5.0800662617338483</v>
+        <v>1</v>
       </c>
       <c r="BL12">
-        <v>0</v>
-      </c>
-      <c r="BM12">
-        <v>2.0581420000000001</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
@@ -3153,10 +3106,10 @@
         <v>2037</v>
       </c>
       <c r="C13">
-        <v>0.10861490122714797</v>
+        <v>3.6024478621328009E-2</v>
       </c>
       <c r="D13">
-        <v>4.6681529289673068E-3</v>
+        <v>9.1156774968811333E-2</v>
       </c>
       <c r="E13">
         <v>1.0184210526315789</v>
@@ -3294,56 +3247,52 @@
         <v>0.25400477788072878</v>
       </c>
       <c r="AX13">
-        <v>1</v>
+        <v>2.1983380000000001</v>
       </c>
       <c r="AY13">
+        <v>0.81646023079441621</v>
+      </c>
+      <c r="AZ13">
+        <v>1</v>
+      </c>
+      <c r="BA13">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ13">
+      <c r="BB13">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA13">
-        <v>0.23201108171109569</v>
-      </c>
-      <c r="BB13">
-        <v>0.16582265327448104</v>
-      </c>
       <c r="BC13">
-        <v>1</v>
+        <v>9.6739499780888316</v>
       </c>
       <c r="BD13">
-        <v>1</v>
+        <v>1.257613497151548E-2</v>
       </c>
       <c r="BE13">
-        <f t="shared" si="0"/>
-        <v>0.13</v>
+        <v>0.1122865976250649</v>
       </c>
       <c r="BF13">
-        <v>0.81646023079441621</v>
+        <v>0.10285922304296979</v>
       </c>
       <c r="BG13">
-        <v>9.6739499780888316</v>
+        <v>5.2054123515665562</v>
       </c>
       <c r="BH13">
-        <v>1.257613497151548E-2</v>
+        <v>5.7239482028646531</v>
       </c>
       <c r="BI13">
-        <v>5.2054123515665562</v>
+        <v>5.4665930425179461</v>
       </c>
       <c r="BJ13">
-        <v>5.7239482028646531</v>
+        <v>8.9453340695748285</v>
       </c>
       <c r="BK13">
-        <v>5.4665930425179461</v>
+        <v>1</v>
       </c>
       <c r="BL13">
-        <v>8.9453340695748285</v>
-      </c>
-      <c r="BM13">
-        <v>2.1983380000000001</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
@@ -3351,10 +3300,10 @@
         <v>2038</v>
       </c>
       <c r="C14">
-        <v>0.1128422052264189</v>
+        <v>3.5462680853742774E-2</v>
       </c>
       <c r="D14">
-        <v>6.5775893466804257E-3</v>
+        <v>0.10274311147919125</v>
       </c>
       <c r="E14">
         <v>1.0152777777777777</v>
@@ -3492,56 +3441,52 @@
         <v>0.26853252711458464</v>
       </c>
       <c r="AX14">
-        <v>1</v>
+        <v>2.3481920000000001</v>
       </c>
       <c r="AY14">
+        <v>0.88493999307285987</v>
+      </c>
+      <c r="AZ14">
+        <v>1</v>
+      </c>
+      <c r="BA14">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ14">
+      <c r="BB14">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA14">
-        <v>0.2468073616929872</v>
-      </c>
-      <c r="BB14">
-        <v>0.17836894596187641</v>
-      </c>
       <c r="BC14">
-        <v>1</v>
+        <v>10.164830005709025</v>
       </c>
       <c r="BD14">
-        <v>1</v>
+        <v>1.3214279007421731E-2</v>
       </c>
       <c r="BE14">
-        <f t="shared" si="0"/>
-        <v>0.14000000000000001</v>
+        <v>0.11953635351507166</v>
       </c>
       <c r="BF14">
-        <v>0.88493999307285987</v>
+        <v>0.11052054574723637</v>
       </c>
       <c r="BG14">
-        <v>10.164830005709025</v>
+        <v>5.5335220946919792</v>
       </c>
       <c r="BH14">
-        <v>1.3214279007421731E-2</v>
+        <v>6.168036383149091</v>
       </c>
       <c r="BI14">
-        <v>5.5335220946919792</v>
+        <v>5.8531198233020429</v>
       </c>
       <c r="BJ14">
-        <v>6.168036383149091</v>
+        <v>9.3318608503589129</v>
       </c>
       <c r="BK14">
-        <v>5.8531198233020429</v>
+        <v>1</v>
       </c>
       <c r="BL14">
-        <v>9.3318608503589129</v>
-      </c>
-      <c r="BM14">
-        <v>2.3481920000000001</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
@@ -3549,10 +3494,10 @@
         <v>2039</v>
       </c>
       <c r="C15">
-        <v>0.11653678253239685</v>
+        <v>3.4900567292005538E-2</v>
       </c>
       <c r="D15">
-        <v>1.0080543293447333E-2</v>
+        <v>0.11419674091706747</v>
       </c>
       <c r="E15">
         <v>1.0117647058823529</v>
@@ -3690,56 +3635,52 @@
         <v>0.28267951373947786</v>
       </c>
       <c r="AX15">
-        <v>1</v>
+        <v>2.5083769999999999</v>
       </c>
       <c r="AY15">
+        <v>0.95348747510453991</v>
+      </c>
+      <c r="AZ15">
+        <v>1</v>
+      </c>
+      <c r="BA15">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ15">
+      <c r="BB15">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA15">
-        <v>0.26139786294867456</v>
-      </c>
-      <c r="BB15">
-        <v>0.19105041509713067</v>
-      </c>
       <c r="BC15">
-        <v>1</v>
+        <v>10.660909127477654</v>
       </c>
       <c r="BD15">
-        <v>1</v>
+        <v>1.385918186572095E-2</v>
       </c>
       <c r="BE15">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.1267016873635588</v>
       </c>
       <c r="BF15">
-        <v>0.95348747510453991</v>
+        <v>0.1182598548637292</v>
       </c>
       <c r="BG15">
-        <v>10.660909127477654</v>
+        <v>5.8563554602224244</v>
       </c>
       <c r="BH15">
-        <v>1.385918186572095E-2</v>
+        <v>6.6173236575819461</v>
       </c>
       <c r="BI15">
-        <v>5.8563554602224244</v>
+        <v>6.2396466040861407</v>
       </c>
       <c r="BJ15">
-        <v>6.6173236575819461</v>
+        <v>9.7183876311430151</v>
       </c>
       <c r="BK15">
-        <v>6.2396466040861407</v>
+        <v>1</v>
       </c>
       <c r="BL15">
-        <v>9.7183876311430151</v>
-      </c>
-      <c r="BM15">
-        <v>2.5083769999999999</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
@@ -3747,10 +3688,10 @@
         <v>2040</v>
       </c>
       <c r="C16">
-        <v>0.11785679828283907</v>
+        <v>3.4338137580891402E-2</v>
       </c>
       <c r="D16">
-        <v>1.3547372385283089E-2</v>
+        <v>0.12552066887844415</v>
       </c>
       <c r="E16">
         <v>1.0078125</v>
@@ -3888,56 +3829,52 @@
         <v>0.36081395669506866</v>
       </c>
       <c r="AX16">
-        <v>1</v>
+        <v>2.6796139999999999</v>
       </c>
       <c r="AY16">
+        <v>1.0221033853022929</v>
+      </c>
+      <c r="AZ16">
+        <v>1</v>
+      </c>
+      <c r="BA16">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ16">
+      <c r="BB16">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA16">
-        <v>0.38830831375828301</v>
-      </c>
-      <c r="BB16">
-        <v>0.2897942670381447</v>
-      </c>
       <c r="BC16">
-        <v>1</v>
+        <v>44.211112865664255</v>
       </c>
       <c r="BD16">
-        <v>1</v>
+        <v>5.7474446725363532E-2</v>
       </c>
       <c r="BE16">
-        <f t="shared" si="0"/>
-        <v>0.16</v>
+        <v>0.17994700051621867</v>
       </c>
       <c r="BF16">
-        <v>1.0221033853022929</v>
+        <v>0.17565053867585262</v>
       </c>
       <c r="BG16">
-        <v>44.211112865664255</v>
+        <v>9.0591875322636675</v>
       </c>
       <c r="BH16">
-        <v>5.7474446725363532E-2</v>
+        <v>10.376702578390177</v>
       </c>
       <c r="BI16">
-        <v>9.0591875322636675</v>
+        <v>9.7228050800662622</v>
       </c>
       <c r="BJ16">
-        <v>10.376702578390177</v>
+        <v>41.07123136388735</v>
       </c>
       <c r="BK16">
-        <v>9.7228050800662622</v>
+        <v>1</v>
       </c>
       <c r="BL16">
-        <v>41.07123136388735</v>
-      </c>
-      <c r="BM16">
-        <v>2.6796139999999999</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
@@ -3945,10 +3882,10 @@
         <v>2041</v>
       </c>
       <c r="C17">
-        <v>0.11862898351136593</v>
+        <v>3.2648947990046487E-2</v>
       </c>
       <c r="D17">
-        <v>1.8685128258673453E-2</v>
+        <v>0.13565679193683688</v>
       </c>
       <c r="E17">
         <v>1.0033333333333332</v>
@@ -4086,56 +4023,52 @@
         <v>0.30988902677401098</v>
       </c>
       <c r="AX17">
-        <v>1</v>
+        <v>2.862673</v>
       </c>
       <c r="AY17">
+        <v>1.0907867488468153</v>
+      </c>
+      <c r="AZ17">
+        <v>1</v>
+      </c>
+      <c r="BA17">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ17">
+      <c r="BB17">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA17">
-        <v>0.28996152928143698</v>
-      </c>
-      <c r="BB17">
-        <v>0.21681888271121572</v>
-      </c>
       <c r="BC17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BE17">
-        <f t="shared" si="0"/>
-        <v>0.17</v>
+        <v>0.14077908893597416</v>
       </c>
       <c r="BF17">
-        <v>1.0907867488468153</v>
+        <v>0.13397243233339365</v>
       </c>
       <c r="BG17">
-        <v>0</v>
+        <v>6.4861930584983849</v>
       </c>
       <c r="BH17">
-        <v>0</v>
+        <v>7.5314954888929098</v>
       </c>
       <c r="BI17">
-        <v>6.4861930584983849</v>
+        <v>7.0127001656543344</v>
       </c>
       <c r="BJ17">
-        <v>7.5314954888929098</v>
+        <v>0</v>
       </c>
       <c r="BK17">
-        <v>7.0127001656543344</v>
+        <v>1</v>
       </c>
       <c r="BL17">
-        <v>0</v>
-      </c>
-      <c r="BM17">
-        <v>2.862673</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
@@ -4143,10 +4076,10 @@
         <v>2042</v>
       </c>
       <c r="C18">
-        <v>0.11889803010665607</v>
+        <v>3.0956900209022309E-2</v>
       </c>
       <c r="D18">
-        <v>2.5335329283573425E-2</v>
+        <v>0.14569120409667749</v>
       </c>
       <c r="E18">
         <v>0.99821428571428583</v>
@@ -4284,56 +4217,52 @@
         <v>0.32298034686891236</v>
       </c>
       <c r="AX18">
-        <v>1</v>
+        <v>3.0583800000000001</v>
       </c>
       <c r="AY18">
+        <v>1.1595383552415865</v>
+      </c>
+      <c r="AZ18">
+        <v>1</v>
+      </c>
+      <c r="BA18">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ18">
+      <c r="BB18">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA18">
-        <v>0.30393469435851117</v>
-      </c>
-      <c r="BB18">
-        <v>0.22990588119004715</v>
-      </c>
       <c r="BC18">
-        <v>1</v>
+        <v>12.180341057674227</v>
       </c>
       <c r="BD18">
-        <v>1</v>
+        <v>1.5834443374976494E-2</v>
       </c>
       <c r="BE18">
-        <f t="shared" si="0"/>
-        <v>0.18</v>
+        <v>0.14769115665990201</v>
       </c>
       <c r="BF18">
-        <v>1.1595383552415865</v>
+        <v>0.14194570068656562</v>
       </c>
       <c r="BG18">
-        <v>12.180341057674227</v>
+        <v>6.7931972912438763</v>
       </c>
       <c r="BH18">
-        <v>1.5834443374976494E-2</v>
+        <v>7.9963800457710414</v>
       </c>
       <c r="BI18">
-        <v>6.7931972912438763</v>
+        <v>7.3992269464384322</v>
       </c>
       <c r="BJ18">
-        <v>7.9963800457710414</v>
+        <v>10.877967973495313</v>
       </c>
       <c r="BK18">
-        <v>7.3992269464384322</v>
+        <v>1</v>
       </c>
       <c r="BL18">
-        <v>10.877967973495313</v>
-      </c>
-      <c r="BM18">
-        <v>3.0583800000000001</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
@@ -4341,10 +4270,10 @@
         <v>2043</v>
       </c>
       <c r="C19">
-        <v>0.11870705510318108</v>
+        <v>2.9261984549030798E-2</v>
       </c>
       <c r="D19">
-        <v>3.3338267909972921E-2</v>
+        <v>0.15562592633076608</v>
       </c>
       <c r="E19">
         <v>0.99230769230769222</v>
@@ -4482,56 +4411,52 @@
         <v>0.3357484061896252</v>
       </c>
       <c r="AX19">
-        <v>1</v>
+        <v>3.267617</v>
       </c>
       <c r="AY19">
+        <v>1.2283572718835276</v>
+      </c>
+      <c r="AZ19">
+        <v>1</v>
+      </c>
+      <c r="BA19">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ19">
+      <c r="BB19">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA19">
-        <v>0.31770208070938211</v>
-      </c>
-      <c r="BB19">
-        <v>0.24312805611673685</v>
-      </c>
       <c r="BC19">
-        <v>1</v>
+        <v>12.697216556036297</v>
       </c>
       <c r="BD19">
-        <v>1</v>
+        <v>1.6506381522847186E-2</v>
       </c>
       <c r="BE19">
-        <f t="shared" si="0"/>
-        <v>0.19</v>
+        <v>0.15451880234231061</v>
       </c>
       <c r="BF19">
-        <v>1.2283572718835276</v>
+        <v>0.14999695545196351</v>
       </c>
       <c r="BG19">
-        <v>12.697216556036297</v>
+        <v>7.094925146394413</v>
       </c>
       <c r="BH19">
-        <v>1.6506381522847186E-2</v>
+        <v>8.4664636967975682</v>
       </c>
       <c r="BI19">
-        <v>7.094925146394413</v>
+        <v>7.785753727222529</v>
       </c>
       <c r="BJ19">
-        <v>8.4664636967975682</v>
+        <v>11.264494754279397</v>
       </c>
       <c r="BK19">
-        <v>7.785753727222529</v>
+        <v>1</v>
       </c>
       <c r="BL19">
-        <v>11.264494754279397</v>
-      </c>
-      <c r="BM19">
-        <v>3.267617</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
@@ -4539,10 +4464,10 @@
         <v>2044</v>
       </c>
       <c r="C20">
-        <v>0.11809786585865492</v>
+        <v>2.7564191271936673E-2</v>
       </c>
       <c r="D20">
-        <v>4.2534991377147384E-2</v>
+        <v>0.16546291996953805</v>
       </c>
       <c r="E20">
         <v>0.98541666666666661</v>
@@ -4680,56 +4605,52 @@
         <v>0.3482072948484029</v>
       </c>
       <c r="AX20">
-        <v>1</v>
+        <v>3.49133</v>
       </c>
       <c r="AY20">
+        <v>1.2972442710025645</v>
+      </c>
+      <c r="AZ20">
+        <v>1</v>
+      </c>
+      <c r="BA20">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ20">
+      <c r="BB20">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA20">
-        <v>0.3312636883340489</v>
-      </c>
-      <c r="BB20">
-        <v>0.25648540749128546</v>
-      </c>
       <c r="BC20">
-        <v>1</v>
+        <v>13.219291148547025</v>
       </c>
       <c r="BD20">
-        <v>1</v>
+        <v>1.7185078493111131E-2</v>
       </c>
       <c r="BE20">
-        <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>0.16126202598319955</v>
       </c>
       <c r="BF20">
-        <v>1.2972442710025645</v>
+        <v>0.15812619662958768</v>
       </c>
       <c r="BG20">
-        <v>13.219291148547025</v>
+        <v>7.3913766239499727</v>
       </c>
       <c r="BH20">
-        <v>1.7185078493111131E-2</v>
+        <v>8.9417464419725139</v>
       </c>
       <c r="BI20">
-        <v>7.3913766239499727</v>
+        <v>8.1722805080066259</v>
       </c>
       <c r="BJ20">
-        <v>8.9417464419725139</v>
+        <v>11.651021535063499</v>
       </c>
       <c r="BK20">
-        <v>8.1722805080066259</v>
+        <v>1</v>
       </c>
       <c r="BL20">
-        <v>11.651021535063499</v>
-      </c>
-      <c r="BM20">
-        <v>3.49133</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
@@ -4737,10 +4658,10 @@
         <v>2045</v>
       </c>
       <c r="C21">
-        <v>0.11601434794570607</v>
+        <v>2.5863510589919373E-2</v>
       </c>
       <c r="D21">
-        <v>5.1720801258956596E-2</v>
+        <v>0.17520408902509096</v>
       </c>
       <c r="E21">
         <v>0.97727272727272729</v>
@@ -4878,56 +4799,52 @@
         <v>0.45970766726296836</v>
       </c>
       <c r="AX21">
-        <v>1</v>
+        <v>3.730531</v>
       </c>
       <c r="AY21">
+        <v>1.3661985358453841</v>
+      </c>
+      <c r="AZ21">
+        <v>1</v>
+      </c>
+      <c r="BA21">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ21">
+      <c r="BB21">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA21">
-        <v>0.53446230940931694</v>
-      </c>
-      <c r="BB21">
-        <v>0.42519911613406625</v>
-      </c>
       <c r="BC21">
-        <v>1</v>
+        <v>73.44701899688819</v>
       </c>
       <c r="BD21">
-        <v>1</v>
+        <v>9.5481124695954642E-2</v>
       </c>
       <c r="BE21">
-        <f t="shared" si="0"/>
-        <v>0.21</v>
+        <v>0.24580505001407876</v>
       </c>
       <c r="BF21">
-        <v>1.3661985358453841</v>
+        <v>0.25588410546196122</v>
       </c>
       <c r="BG21">
-        <v>73.44701899688819</v>
+        <v>12.550315625879922</v>
       </c>
       <c r="BH21">
-        <v>9.5481124695954642E-2</v>
+        <v>15.392273697464081</v>
       </c>
       <c r="BI21">
-        <v>12.550315625879922</v>
+        <v>13.981778023191607</v>
       </c>
       <c r="BJ21">
-        <v>15.392273697464081</v>
+        <v>66.267255659856431</v>
       </c>
       <c r="BK21">
-        <v>13.981778023191607</v>
+        <v>1</v>
       </c>
       <c r="BL21">
-        <v>66.267255659856431</v>
-      </c>
-      <c r="BM21">
-        <v>3.730531</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
@@ -4935,10 +4852,10 @@
         <v>2046</v>
       </c>
       <c r="C22">
-        <v>0.11601434794570607</v>
+        <v>2.2453447609377328E-2</v>
       </c>
       <c r="D22">
-        <v>5.1720801258956596E-2</v>
+        <v>0.18282801413575031</v>
       </c>
       <c r="E22">
         <v>0.96749999999999992</v>
@@ -5076,56 +4993,52 @@
         <v>0.37225294979311929</v>
       </c>
       <c r="AX22">
-        <v>1</v>
+        <v>3.9863029999999999</v>
       </c>
       <c r="AY22">
+        <v>1.4352204684295875</v>
+      </c>
+      <c r="AZ22">
+        <v>1</v>
+      </c>
+      <c r="BA22">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ22">
+      <c r="BB22">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA22">
-        <v>0.35776956740476945</v>
-      </c>
-      <c r="BB22">
-        <v>0.28360563958395973</v>
-      </c>
       <c r="BC22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BE22">
-        <f t="shared" si="0"/>
-        <v>0.22</v>
+        <v>0.17449520714041827</v>
       </c>
       <c r="BF22">
-        <v>1.4352204684295875</v>
+        <v>0.17461863822151516</v>
       </c>
       <c r="BG22">
-        <v>0</v>
+        <v>7.9684504462761403</v>
       </c>
       <c r="BH22">
-        <v>0</v>
+        <v>9.9079092147676775</v>
       </c>
       <c r="BI22">
-        <v>7.9684504462761403</v>
+        <v>8.9453340695748214</v>
       </c>
       <c r="BJ22">
-        <v>9.9079092147676775</v>
+        <v>0</v>
       </c>
       <c r="BK22">
-        <v>8.9453340695748214</v>
+        <v>1</v>
       </c>
       <c r="BL22">
-        <v>0</v>
-      </c>
-      <c r="BM22">
-        <v>3.9863029999999999</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
@@ -5133,10 +5046,10 @@
         <v>2047</v>
       </c>
       <c r="C23">
-        <v>0.11601434794570607</v>
+        <v>1.9031716298215918E-2</v>
       </c>
       <c r="D23">
-        <v>5.1720801258956596E-2</v>
+        <v>0.19039425451906636</v>
       </c>
       <c r="E23">
         <v>0.9555555555555556</v>
@@ -5274,56 +5187,52 @@
         <v>0.38386683556126833</v>
       </c>
       <c r="AX23">
-        <v>1</v>
+        <v>4.2598079999999996</v>
       </c>
       <c r="AY23">
+        <v>1.5043098142096942</v>
+      </c>
+      <c r="AZ23">
+        <v>1</v>
+      </c>
+      <c r="BA23">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ23">
+      <c r="BB23">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA23">
-        <v>0.37071383885082393</v>
-      </c>
-      <c r="BB23">
-        <v>0.29736852030208494</v>
-      </c>
       <c r="BC23">
-        <v>1</v>
+        <v>14.816709490969675</v>
       </c>
       <c r="BD23">
-        <v>1</v>
+        <v>1.9261722338260578E-2</v>
       </c>
       <c r="BE23">
-        <f t="shared" si="0"/>
-        <v>0.23</v>
+        <v>0.1809851646567483</v>
       </c>
       <c r="BF23">
-        <v>1.5043098142096942</v>
+        <v>0.18298183863581816</v>
       </c>
       <c r="BG23">
-        <v>14.816709490969675</v>
+        <v>8.2490727910467676</v>
       </c>
       <c r="BH23">
-        <v>1.9261722338260578E-2</v>
+        <v>10.398789242387878</v>
       </c>
       <c r="BI23">
-        <v>8.2490727910467676</v>
+        <v>9.3318608503589182</v>
       </c>
       <c r="BJ23">
-        <v>10.398789242387878</v>
+        <v>12.810601877415788</v>
       </c>
       <c r="BK23">
-        <v>9.3318608503589182</v>
+        <v>1</v>
       </c>
       <c r="BL23">
-        <v>12.810601877415788</v>
-      </c>
-      <c r="BM23">
-        <v>4.2598079999999996</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
@@ -5331,10 +5240,10 @@
         <v>2048</v>
       </c>
       <c r="C24">
-        <v>0.11601434794570607</v>
+        <v>1.5598236530324307E-2</v>
       </c>
       <c r="D24">
-        <v>5.1720801258956596E-2</v>
+        <v>0.1979036765411975</v>
       </c>
       <c r="E24">
         <v>0.94062500000000004</v>
@@ -5472,56 +5381,52 @@
         <v>0.39522573724306265</v>
       </c>
       <c r="AX24">
-        <v>1</v>
+        <v>4.5522869999999998</v>
       </c>
       <c r="AY24">
+        <v>1.5734666341443346</v>
+      </c>
+      <c r="AZ24">
+        <v>1</v>
+      </c>
+      <c r="BA24">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ24">
+      <c r="BB24">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA24">
-        <v>0.38345233157067432</v>
-      </c>
-      <c r="BB24">
-        <v>0.31126657746806891</v>
-      </c>
       <c r="BC24">
-        <v>1</v>
+        <v>15.359580460074014</v>
       </c>
       <c r="BD24">
-        <v>1</v>
+        <v>1.9967454598096217E-2</v>
       </c>
       <c r="BE24">
-        <f t="shared" si="0"/>
-        <v>0.24</v>
+        <v>0.18739070013155873</v>
       </c>
       <c r="BF24">
-        <v>1.5734666341443346</v>
+        <v>0.19142302546234738</v>
       </c>
       <c r="BG24">
-        <v>15.359580460074014</v>
+        <v>8.5244187582224189</v>
       </c>
       <c r="BH24">
-        <v>1.9967454598096217E-2</v>
+        <v>10.894868364156492</v>
       </c>
       <c r="BI24">
-        <v>8.5244187582224189</v>
+        <v>9.7183876311430151</v>
       </c>
       <c r="BJ24">
-        <v>10.894868364156492</v>
+        <v>13.19712865819989</v>
       </c>
       <c r="BK24">
-        <v>9.7183876311430151</v>
+        <v>1</v>
       </c>
       <c r="BL24">
-        <v>13.19712865819989</v>
-      </c>
-      <c r="BM24">
-        <v>4.5522869999999998</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
@@ -5529,10 +5434,10 @@
         <v>2049</v>
       </c>
       <c r="C25">
-        <v>0.11601434794570607</v>
+        <v>1.2152927351411538E-2</v>
       </c>
       <c r="D25">
-        <v>5.1720801258956596E-2</v>
+        <v>0.20535712719577859</v>
       </c>
       <c r="E25">
         <v>0.92142857142857126</v>
@@ -5670,56 +5575,52 @@
         <v>0.40634252685002109</v>
       </c>
       <c r="AX25">
-        <v>1</v>
+        <v>4.8650700000000002</v>
       </c>
       <c r="AY25">
+        <v>1.6426906603487994</v>
+      </c>
+      <c r="AZ25">
+        <v>1</v>
+      </c>
+      <c r="BA25">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ25">
+      <c r="BB25">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA25">
-        <v>0.39598504556431974</v>
-      </c>
-      <c r="BB25">
-        <v>0.3252998110819123</v>
-      </c>
       <c r="BC25">
-        <v>1</v>
+        <v>15.907650523327064</v>
       </c>
       <c r="BD25">
-        <v>1</v>
+        <v>2.0679945680325183E-2</v>
       </c>
       <c r="BE25">
-        <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.19371181356484912</v>
       </c>
       <c r="BF25">
-        <v>1.6426906603487994</v>
+        <v>0.19994219870110322</v>
       </c>
       <c r="BG25">
-        <v>15.907650523327064</v>
+        <v>8.7944883478030711</v>
       </c>
       <c r="BH25">
-        <v>2.0679945680325183E-2</v>
+        <v>11.396146580073548</v>
       </c>
       <c r="BI25">
-        <v>8.7944883478030711</v>
+        <v>10.104914411927112</v>
       </c>
       <c r="BJ25">
-        <v>11.396146580073548</v>
+        <v>13.583655438983975</v>
       </c>
       <c r="BK25">
-        <v>10.104914411927112</v>
+        <v>1</v>
       </c>
       <c r="BL25">
-        <v>13.583655438983975</v>
-      </c>
-      <c r="BM25">
-        <v>4.8650700000000002</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:65" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
@@ -5727,10 +5628,10 @@
         <v>2050</v>
       </c>
       <c r="C26">
-        <v>0.11601434794570607</v>
+        <v>8.695706967553913E-3</v>
       </c>
       <c r="D26">
-        <v>5.1720801258956596E-2</v>
+        <v>0.21275543467722335</v>
       </c>
       <c r="E26">
         <v>0.89583333333333337</v>
@@ -5868,53 +5769,49 @@
         <v>0.49043108014036285</v>
       </c>
       <c r="AX26">
-        <v>0</v>
+        <v>5.1995820000000004</v>
       </c>
       <c r="AY26">
+        <v>1.7119816847925917</v>
+      </c>
+      <c r="AZ26">
+        <v>0</v>
+      </c>
+      <c r="BA26">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AZ26">
+      <c r="BB26">
         <v>-3.8381578947368399E-2</v>
       </c>
-      <c r="BA26">
-        <v>0.56700484632745951</v>
-      </c>
-      <c r="BB26">
-        <v>0.47846831584043548</v>
-      </c>
       <c r="BC26">
-        <v>1</v>
+        <v>69.922494564120896</v>
       </c>
       <c r="BD26">
-        <v>1</v>
+        <v>9.0899242933357161E-2</v>
       </c>
       <c r="BE26">
-        <f t="shared" si="0"/>
-        <v>0.26</v>
+        <v>0.26505327028818854</v>
       </c>
       <c r="BF26">
-        <v>1.7119816847925917</v>
+        <v>0.28873172067717423</v>
       </c>
       <c r="BG26">
-        <v>69.922494564120896</v>
+        <v>13.128329393011782</v>
       </c>
       <c r="BH26">
-        <v>9.0899242933357161E-2</v>
+        <v>17.248781378478281</v>
       </c>
       <c r="BI26">
-        <v>13.128329393011782</v>
+        <v>15.20375483158476</v>
       </c>
       <c r="BJ26">
-        <v>17.248781378478281</v>
+        <v>61.093318608503587</v>
       </c>
       <c r="BK26">
-        <v>15.20375483158476</v>
+        <v>1</v>
       </c>
       <c r="BL26">
-        <v>61.093318608503587</v>
-      </c>
-      <c r="BM26">
-        <v>5.1995820000000004</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>